<commit_message>
fix(productos): Fase A — kits Excel v1.1 (escandallos, APPCC, inventario, gestión de personal, plan financiero): 57 xlsx con cache de valores, A4, metadata AI Chef Pro, bio anclada, línea de versión; calculadora PVP reparada (9 fórmulas '=…/=AVERAGE' → '/AVERAGE')
Co-Authored-By: Claude Fable 5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_016924EP7QJuq6BNFj8S7Fks
</commit_message>
<xml_diff>
--- a/astro-site/public/dl/kit-escandallos/01-escandallo-estandar.xlsx
+++ b/astro-site/public/dl/kit-escandallos/01-escandallo-estandar.xlsx
@@ -1,17 +1,18 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr/>
   <workbookProtection/>
   <bookViews>
-    <workbookView activeTab="0" autoFilterDateGrouping="1" firstSheet="0" minimized="0" showHorizontalScroll="1" showSheetTabs="1" showVerticalScroll="1" tabRatio="600" visibility="visible"/>
+    <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet name="Instrucciones" sheetId="1" state="visible" r:id="rId1"/>
-    <sheet name="Escandallo" sheetId="2" state="visible" r:id="rId2"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Instrucciones" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Escandallo" sheetId="2" state="visible" r:id="rId2"/>
   </sheets>
   <definedNames>
-    <definedName localSheetId="1" name="_xlnm.Print_Area">'Escandallo'!$A$1:$I$29</definedName>
+    <definedName name="_xlnm.Print_Titles" localSheetId="1">'Escandallo'!$4:$4</definedName>
+    <definedName name="_xlnm.Print_Area" localSheetId="1">'Escandallo'!$A$1:$I$29</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -20,9 +21,9 @@
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <numFmts count="3">
-    <numFmt formatCode="#,##0.00 €" numFmtId="164"/>
-    <numFmt formatCode="0.000" numFmtId="165"/>
-    <numFmt formatCode="0.0%" numFmtId="166"/>
+    <numFmt numFmtId="164" formatCode="#,##0.00 €"/>
+    <numFmt numFmtId="165" formatCode="0.000"/>
+    <numFmt numFmtId="166" formatCode="0.0%"/>
   </numFmts>
   <fonts count="18">
     <font>
@@ -167,7 +168,7 @@
       </patternFill>
     </fill>
   </fills>
-  <borders count="15">
+  <borders count="20">
     <border>
       <left/>
       <right/>
@@ -347,112 +348,172 @@
         <color rgb="00E0E0E0"/>
       </bottom>
     </border>
+    <border>
+      <left/>
+      <right/>
+      <top style="thin">
+        <color rgb="00E0E0E0"/>
+      </top>
+      <bottom style="thin">
+        <color rgb="00E0E0E0"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right style="thin">
+        <color rgb="00E0E0E0"/>
+      </right>
+      <top style="thin">
+        <color rgb="00E0E0E0"/>
+      </top>
+      <bottom style="thin">
+        <color rgb="00E0E0E0"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right/>
+      <top style="medium">
+        <color rgb="00FFD700"/>
+      </top>
+      <bottom/>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right style="medium">
+        <color rgb="00FFD700"/>
+      </right>
+      <top style="medium">
+        <color rgb="00FFD700"/>
+      </top>
+      <bottom/>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right style="medium">
+        <color rgb="00FFD700"/>
+      </right>
+      <top style="medium">
+        <color rgb="00FFD700"/>
+      </top>
+      <bottom style="medium">
+        <color rgb="00FFD700"/>
+      </bottom>
+      <diagonal/>
+    </border>
   </borders>
   <cellStyleXfs count="1">
-    <xf borderId="0" fillId="0" fontId="0" numFmtId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="48">
-    <xf borderId="0" fillId="0" fontId="0" numFmtId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf applyAlignment="1" borderId="0" fillId="0" fontId="1" numFmtId="0" pivotButton="0" quotePrefix="0" xfId="0">
+  <cellXfs count="51">
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
-    <xf borderId="0" fillId="0" fontId="2" numFmtId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf borderId="0" fillId="0" fontId="3" numFmtId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf applyAlignment="1" borderId="0" fillId="0" fontId="4" numFmtId="0" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="top" wrapText="1"/>
     </xf>
-    <xf applyAlignment="1" borderId="0" fillId="0" fontId="0" numFmtId="0" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="top" wrapText="1"/>
     </xf>
-    <xf applyAlignment="1" borderId="0" fillId="0" fontId="5" numFmtId="0" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="top" wrapText="1"/>
     </xf>
-    <xf applyAlignment="1" borderId="0" fillId="0" fontId="6" numFmtId="0" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="top" wrapText="1"/>
     </xf>
-    <xf borderId="0" fillId="0" fontId="7" numFmtId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf applyAlignment="1" borderId="0" fillId="0" fontId="11" numFmtId="0" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="11" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
-    <xf applyAlignment="1" borderId="1" fillId="0" fontId="8" numFmtId="0" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="8" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf borderId="1" fillId="0" fontId="0" numFmtId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf applyAlignment="1" borderId="14" fillId="3" fontId="12" numFmtId="0" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="12" fillId="3" borderId="14" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf borderId="2" fillId="2" fontId="0" numFmtId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf borderId="3" fillId="2" fontId="0" numFmtId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf applyAlignment="1" borderId="14" fillId="4" fontId="5" numFmtId="0" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="0" fillId="2" borderId="2" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="2" borderId="3" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="5" fillId="4" borderId="14" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
-    <xf applyAlignment="1" borderId="14" fillId="4" fontId="5" numFmtId="0" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="5" fillId="4" borderId="14" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf applyAlignment="1" borderId="14" fillId="4" fontId="5" numFmtId="164" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="164" fontId="5" fillId="4" borderId="14" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="right" vertical="center"/>
     </xf>
-    <xf applyAlignment="1" borderId="14" fillId="4" fontId="5" numFmtId="165" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="165" fontId="5" fillId="4" borderId="14" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="right" vertical="center"/>
     </xf>
-    <xf applyAlignment="1" borderId="14" fillId="4" fontId="5" numFmtId="9" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="9" fontId="5" fillId="4" borderId="14" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf applyAlignment="1" borderId="14" fillId="0" fontId="13" numFmtId="165" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="165" fontId="13" fillId="0" borderId="14" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="right" vertical="center"/>
     </xf>
-    <xf applyAlignment="1" borderId="14" fillId="0" fontId="13" numFmtId="164" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="164" fontId="13" fillId="0" borderId="14" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="right" vertical="center"/>
     </xf>
-    <xf borderId="4" fillId="2" fontId="0" numFmtId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf borderId="5" fillId="2" fontId="0" numFmtId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf applyAlignment="1" borderId="4" fillId="2" fontId="9" numFmtId="0" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="0" fillId="2" borderId="4" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="2" borderId="5" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="9" fillId="2" borderId="4" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf borderId="10" fillId="0" fontId="0" numFmtId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf borderId="12" fillId="0" fontId="0" numFmtId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf borderId="13" fillId="0" fontId="0" numFmtId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf borderId="6" fillId="2" fontId="0" numFmtId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf borderId="7" fillId="2" fontId="0" numFmtId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf borderId="14" fillId="4" fontId="0" numFmtId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf borderId="14" fillId="4" fontId="0" numFmtId="9" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf borderId="14" fillId="0" fontId="0" numFmtId="165" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf borderId="14" fillId="0" fontId="0" numFmtId="164" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf applyAlignment="1" borderId="0" fillId="0" fontId="10" numFmtId="0" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="10" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="12" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="13" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="2" borderId="6" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="2" borderId="7" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="4" borderId="14" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="9" fontId="0" fillId="4" borderId="14" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="165" fontId="0" fillId="0" borderId="14" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="164" fontId="0" fillId="0" borderId="14" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="10" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf applyAlignment="1" borderId="14" fillId="5" fontId="4" numFmtId="0" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="4" fillId="5" borderId="14" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="right" vertical="center"/>
     </xf>
-    <xf borderId="14" fillId="5" fontId="4" numFmtId="164" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf applyAlignment="1" borderId="14" fillId="0" fontId="5" numFmtId="0" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="164" fontId="4" fillId="5" borderId="14" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="14" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="right" vertical="center"/>
     </xf>
-    <xf borderId="14" fillId="0" fontId="13" numFmtId="164" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf applyAlignment="1" borderId="14" fillId="6" fontId="14" numFmtId="0" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="164" fontId="13" fillId="0" borderId="14" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="14" fillId="6" borderId="14" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="right" vertical="center"/>
     </xf>
-    <xf borderId="14" fillId="6" fontId="15" numFmtId="164" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf applyAlignment="1" borderId="14" fillId="0" fontId="13" numFmtId="0" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="164" fontId="15" fillId="6" borderId="14" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="13" fillId="0" borderId="14" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="right" vertical="center"/>
     </xf>
-    <xf applyAlignment="1" borderId="14" fillId="4" fontId="16" numFmtId="9" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="9" fontId="16" fillId="4" borderId="14" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf applyAlignment="1" borderId="14" fillId="0" fontId="4" numFmtId="0" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="14" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="right" vertical="center"/>
     </xf>
-    <xf borderId="14" fillId="0" fontId="4" numFmtId="164" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf applyAlignment="1" borderId="14" fillId="6" fontId="4" numFmtId="0" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="164" fontId="4" fillId="0" borderId="14" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="4" fillId="6" borderId="14" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="right" vertical="center"/>
     </xf>
-    <xf borderId="14" fillId="6" fontId="17" numFmtId="164" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf borderId="14" fillId="0" fontId="13" numFmtId="166" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="164" fontId="17" fillId="6" borderId="14" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="166" fontId="13" fillId="0" borderId="14" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="19" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="15" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="16" pivotButton="0" quotePrefix="0" xfId="0"/>
   </cellXfs>
   <cellStyles count="1">
-    <cellStyle builtinId="0" hidden="0" name="Normal" xfId="0"/>
+    <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
   </cellStyles>
-  <tableStyles count="0" defaultPivotStyle="PivotStyleLight16" defaultTableStyle="TableStyleMedium9"/>
+  <tableStyles count="0" defaultTableStyle="TableStyleMedium9" defaultPivotStyle="PivotStyleLight16"/>
   <colors>
     <indexedColors>
       <rgbColor rgb="00000000"/>
@@ -812,15 +873,16 @@
   <sheetPr>
     <tabColor rgb="00FFD700"/>
     <outlinePr summaryBelow="1" summaryRight="1"/>
-    <pageSetUpPr/>
+    <pageSetUpPr fitToPage="1"/>
   </sheetPr>
-  <dimension ref="B2:B34"/>
+  <dimension ref="A1:B36"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
-    <col customWidth="1" max="1" min="1" width="3"/>
-    <col customWidth="1" max="2" min="2" width="80"/>
+    <col width="3" customWidth="1" min="1" max="1"/>
+    <col width="80" customWidth="1" min="2" max="2"/>
   </cols>
   <sheetData>
+    <row r="1"/>
     <row r="2">
       <c r="B2" s="1" t="inlineStr">
         <is>
@@ -842,6 +904,7 @@
         </is>
       </c>
     </row>
+    <row r="5"/>
     <row r="6">
       <c r="B6" s="4" t="inlineStr">
         <is>
@@ -1007,10 +1070,19 @@
         </is>
       </c>
     </row>
+    <row r="33"/>
     <row r="34">
       <c r="B34" s="8" t="inlineStr">
         <is>
           <t>© 2026 AI Chef Pro · Todos los derechos reservados</t>
+        </is>
+      </c>
+    </row>
+    <row r="35"/>
+    <row r="36">
+      <c r="B36" s="8" t="inlineStr">
+        <is>
+          <t>Versión 1.1 · agosto 2026 · aichef.pro/kit-escandallos · info@aichef.pro</t>
         </is>
       </c>
     </row>
@@ -1018,7 +1090,16 @@
   <mergeCells count="1">
     <mergeCell ref="B2"/>
   </mergeCells>
-  <pageMargins bottom="1" footer="0.5" header="0.5" left="0.75" right="0.75" top="1"/>
+  <pageMargins left="0.59" right="0.59" top="0.59" bottom="0.59" header="0.3" footer="0.3"/>
+  <pageSetup orientation="portrait" paperSize="9" fitToHeight="0" fitToWidth="1"/>
+  <headerFooter>
+    <oddHeader/>
+    <oddFooter>&amp;C&amp;8 AI Chef Pro · aichef.pro · Página &amp;P de &amp;N</oddFooter>
+    <evenHeader/>
+    <evenFooter/>
+    <firstHeader/>
+    <firstFooter/>
+  </headerFooter>
 </worksheet>
 </file>
 
@@ -1027,23 +1108,23 @@
   <sheetPr>
     <tabColor rgb="00FFD700"/>
     <outlinePr summaryBelow="1" summaryRight="1"/>
-    <pageSetUpPr/>
+    <pageSetUpPr fitToPage="1"/>
   </sheetPr>
   <dimension ref="A1:L29"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
-    <col customWidth="1" max="1" min="1" width="25"/>
-    <col customWidth="1" max="2" min="2" width="16"/>
-    <col customWidth="1" max="3" min="3" width="12"/>
-    <col customWidth="1" max="4" min="4" width="14"/>
-    <col customWidth="1" max="5" min="5" width="12"/>
-    <col customWidth="1" max="6" min="6" width="12"/>
-    <col customWidth="1" max="7" min="7" width="10"/>
-    <col customWidth="1" max="8" min="8" width="14"/>
-    <col customWidth="1" max="9" min="9" width="14"/>
-    <col customWidth="1" max="10" min="10" width="3"/>
-    <col customWidth="1" max="11" min="11" width="20"/>
-    <col customWidth="1" max="12" min="12" width="20"/>
+    <col width="25" customWidth="1" min="1" max="1"/>
+    <col width="16" customWidth="1" min="2" max="2"/>
+    <col width="12" customWidth="1" min="3" max="3"/>
+    <col width="14" customWidth="1" min="4" max="4"/>
+    <col width="12" customWidth="1" min="5" max="5"/>
+    <col width="12" customWidth="1" min="6" max="6"/>
+    <col width="10" customWidth="1" min="7" max="7"/>
+    <col width="14" customWidth="1" min="8" max="8"/>
+    <col width="14" customWidth="1" min="9" max="9"/>
+    <col width="3" customWidth="1" min="10" max="10"/>
+    <col width="20" customWidth="1" min="11" max="11"/>
+    <col width="20" customWidth="1" min="12" max="12"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -1066,7 +1147,7 @@
           <t>📷 Foto del Plato</t>
         </is>
       </c>
-      <c r="L3" s="11" t="n"/>
+      <c r="L3" s="48" t="n"/>
     </row>
     <row r="4">
       <c r="A4" s="12" t="inlineStr">
@@ -1149,11 +1230,11 @@
       </c>
       <c r="H5" s="20">
         <f>E5/(1-G5)</f>
-        <v/>
+        <v>0.25</v>
       </c>
       <c r="I5" s="21">
         <f>H5*D5</f>
-        <v/>
+        <v>7.125</v>
       </c>
       <c r="K5" s="22" t="n"/>
       <c r="L5" s="23" t="n"/>
@@ -1190,11 +1271,11 @@
       </c>
       <c r="H6" s="20">
         <f>E6/(1-G6)</f>
-        <v/>
+        <v>0.17045454545454544</v>
       </c>
       <c r="I6" s="21">
         <f>H6*D6</f>
-        <v/>
+        <v>0.3068181818181818</v>
       </c>
       <c r="K6" s="22" t="n"/>
       <c r="L6" s="23" t="n"/>
@@ -1231,11 +1312,11 @@
       </c>
       <c r="H7" s="20">
         <f>E7/(1-G7)</f>
-        <v/>
+        <v>0.10666666666666667</v>
       </c>
       <c r="I7" s="21">
         <f>H7*D7</f>
-        <v/>
+        <v>0.6933333333333334</v>
       </c>
       <c r="K7" s="22" t="n"/>
       <c r="L7" s="23" t="n"/>
@@ -1272,11 +1353,11 @@
       </c>
       <c r="H8" s="20">
         <f>E8/(1-G8)</f>
-        <v/>
+        <v>0.030927835051546393</v>
       </c>
       <c r="I8" s="21">
         <f>H8*D8</f>
-        <v/>
+        <v>0.27835051546391754</v>
       </c>
       <c r="K8" s="24" t="inlineStr">
         <is>
@@ -1318,11 +1399,11 @@
       </c>
       <c r="H9" s="20">
         <f>E9/(1-G9)</f>
-        <v/>
+        <v>0.05102040816326531</v>
       </c>
       <c r="I9" s="21">
         <f>H9*D9</f>
-        <v/>
+        <v>0.4336734693877551</v>
       </c>
       <c r="K9" s="26" t="n"/>
       <c r="L9" s="27" t="n"/>
@@ -1359,11 +1440,11 @@
       </c>
       <c r="H10" s="20">
         <f>E10/(1-G10)</f>
-        <v/>
+        <v>0.08602150537634409</v>
       </c>
       <c r="I10" s="21">
         <f>H10*D10</f>
-        <v/>
+        <v>1.032258064516129</v>
       </c>
       <c r="K10" s="22" t="n"/>
       <c r="L10" s="23" t="n"/>
@@ -1400,11 +1481,11 @@
       </c>
       <c r="H11" s="20">
         <f>E11/(1-G11)</f>
-        <v/>
+        <v>0.030927835051546393</v>
       </c>
       <c r="I11" s="21">
         <f>H11*D11</f>
-        <v/>
+        <v>0.23195876288659795</v>
       </c>
       <c r="K11" s="22" t="n"/>
       <c r="L11" s="23" t="n"/>
@@ -1441,11 +1522,11 @@
       </c>
       <c r="H12" s="20">
         <f>E12/(1-G12)</f>
-        <v/>
+        <v>0.0030612244897959186</v>
       </c>
       <c r="I12" s="21">
         <f>H12*D12</f>
-        <v/>
+        <v>0.04591836734693878</v>
       </c>
       <c r="K12" s="22" t="n"/>
       <c r="L12" s="23" t="n"/>
@@ -1482,11 +1563,11 @@
       </c>
       <c r="H13" s="20">
         <f>E13/(1-G13)</f>
-        <v/>
+        <v>0.0025</v>
       </c>
       <c r="I13" s="21">
         <f>H13*D13</f>
-        <v/>
+        <v>0.0625</v>
       </c>
       <c r="K13" s="22" t="n"/>
       <c r="L13" s="23" t="n"/>
@@ -1523,11 +1604,11 @@
       </c>
       <c r="H14" s="20">
         <f>E14/(1-G14)</f>
-        <v/>
+        <v>1.1111111111111112</v>
       </c>
       <c r="I14" s="21">
         <f>H14*D14</f>
-        <v/>
+        <v>3.8888888888888893</v>
       </c>
       <c r="K14" s="28" t="n"/>
       <c r="L14" s="29" t="n"/>
@@ -1622,15 +1703,23 @@
         <v/>
       </c>
     </row>
+    <row r="20"/>
     <row r="21">
       <c r="A21" s="35" t="inlineStr">
         <is>
           <t>COSTE TOTAL INGREDIENTES</t>
         </is>
       </c>
+      <c r="B21" s="49" t="n"/>
+      <c r="C21" s="49" t="n"/>
+      <c r="D21" s="49" t="n"/>
+      <c r="E21" s="49" t="n"/>
+      <c r="F21" s="49" t="n"/>
+      <c r="G21" s="49" t="n"/>
+      <c r="H21" s="50" t="n"/>
       <c r="I21" s="36">
         <f>SUM(I5:I19)</f>
-        <v/>
+        <v>14.098699583641741</v>
       </c>
     </row>
     <row r="22">
@@ -1639,12 +1728,18 @@
           <t>Coste elaboración (%)</t>
         </is>
       </c>
+      <c r="B22" s="49" t="n"/>
+      <c r="C22" s="49" t="n"/>
+      <c r="D22" s="49" t="n"/>
+      <c r="E22" s="49" t="n"/>
+      <c r="F22" s="49" t="n"/>
+      <c r="G22" s="50" t="n"/>
       <c r="H22" s="19" t="n">
         <v>0.1</v>
       </c>
       <c r="I22" s="38">
         <f>I21*H22</f>
-        <v/>
+        <v>1.4098699583641743</v>
       </c>
     </row>
     <row r="23">
@@ -1653,17 +1748,31 @@
           <t>COSTE TOTAL DEL PLATO</t>
         </is>
       </c>
+      <c r="B23" s="49" t="n"/>
+      <c r="C23" s="49" t="n"/>
+      <c r="D23" s="49" t="n"/>
+      <c r="E23" s="49" t="n"/>
+      <c r="F23" s="49" t="n"/>
+      <c r="G23" s="49" t="n"/>
+      <c r="H23" s="50" t="n"/>
       <c r="I23" s="40">
         <f>I21+I22</f>
-        <v/>
-      </c>
-    </row>
+        <v>15.508569542005915</v>
+      </c>
+    </row>
+    <row r="24"/>
     <row r="25">
       <c r="A25" s="41" t="inlineStr">
         <is>
           <t>Food Cost objetivo (%)</t>
         </is>
       </c>
+      <c r="B25" s="49" t="n"/>
+      <c r="C25" s="49" t="n"/>
+      <c r="D25" s="49" t="n"/>
+      <c r="E25" s="49" t="n"/>
+      <c r="F25" s="49" t="n"/>
+      <c r="G25" s="50" t="n"/>
       <c r="H25" s="42" t="n">
         <v>0.3</v>
       </c>
@@ -1674,9 +1783,16 @@
           <t>PVP SUGERIDO (sin IVA)</t>
         </is>
       </c>
+      <c r="B26" s="49" t="n"/>
+      <c r="C26" s="49" t="n"/>
+      <c r="D26" s="49" t="n"/>
+      <c r="E26" s="49" t="n"/>
+      <c r="F26" s="49" t="n"/>
+      <c r="G26" s="49" t="n"/>
+      <c r="H26" s="50" t="n"/>
       <c r="I26" s="44">
         <f>I23/H25</f>
-        <v/>
+        <v>51.69523180668639</v>
       </c>
     </row>
     <row r="27">
@@ -1685,9 +1801,16 @@
           <t>PVP CON IVA (10% hostelería)</t>
         </is>
       </c>
+      <c r="B27" s="49" t="n"/>
+      <c r="C27" s="49" t="n"/>
+      <c r="D27" s="49" t="n"/>
+      <c r="E27" s="49" t="n"/>
+      <c r="F27" s="49" t="n"/>
+      <c r="G27" s="49" t="n"/>
+      <c r="H27" s="50" t="n"/>
       <c r="I27" s="46">
         <f>I26*1.10</f>
-        <v/>
+        <v>56.86475498735503</v>
       </c>
     </row>
     <row r="28">
@@ -1696,9 +1819,16 @@
           <t>Margen bruto (€)</t>
         </is>
       </c>
+      <c r="B28" s="49" t="n"/>
+      <c r="C28" s="49" t="n"/>
+      <c r="D28" s="49" t="n"/>
+      <c r="E28" s="49" t="n"/>
+      <c r="F28" s="49" t="n"/>
+      <c r="G28" s="49" t="n"/>
+      <c r="H28" s="50" t="n"/>
       <c r="I28" s="38">
         <f>I26-I23</f>
-        <v/>
+        <v>36.18666226468047</v>
       </c>
     </row>
     <row r="29">
@@ -1707,9 +1837,16 @@
           <t>Margen bruto (%)</t>
         </is>
       </c>
+      <c r="B29" s="49" t="n"/>
+      <c r="C29" s="49" t="n"/>
+      <c r="D29" s="49" t="n"/>
+      <c r="E29" s="49" t="n"/>
+      <c r="F29" s="49" t="n"/>
+      <c r="G29" s="49" t="n"/>
+      <c r="H29" s="50" t="n"/>
       <c r="I29" s="47">
         <f>I28/I26</f>
-        <v/>
+        <v>0.7000000000000001</v>
       </c>
     </row>
   </sheetData>
@@ -1729,14 +1866,22 @@
     <mergeCell ref="A22:G22"/>
   </mergeCells>
   <dataValidations count="2">
-    <dataValidation allowBlank="1" error="Selecciona una categoría válida" errorTitle="Categoría inválida" showDropDown="0" showErrorMessage="0" showInputMessage="0" sqref="B5 B6 B7 B8 B9 B10 B11 B12 B13 B14 B15 B16 B17 B18 B19" type="list">
+    <dataValidation sqref="B5 B6 B7 B8 B9 B10 B11 B12 B13 B14 B15 B16 B17 B18 B19" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" errorTitle="Categoría inválida" error="Selecciona una categoría válida" type="list">
       <formula1>"Carne roja,Aves,Pescado,Marisco,Verdura hoja,Verdura raíz,Fruta,Lácteos,Secos/granos,Congelados,Pan/bollería,Huevos,Aceites/grasas,Especias/hierbas,Chocolate/cacao,Bebidas/licores"</formula1>
     </dataValidation>
-    <dataValidation allowBlank="1" showDropDown="0" showErrorMessage="0" showInputMessage="0" sqref="C5 C6 C7 C8 C9 C10 C11 C12 C13 C14 C15 C16 C17 C18 C19 F5 F6 F7 F8 F9 F10 F11 F12 F13 F14 F15 F16 F17 F18 F19" type="list">
+    <dataValidation sqref="C5 C6 C7 C8 C9 C10 C11 C12 C13 C14 C15 C16 C17 C18 C19 F5 F6 F7 F8 F9 F10 F11 F12 F13 F14 F15 F16 F17 F18 F19" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
       <formula1>"kg,g,L,ml,cl,ud,docena,manojo,sobre,lata,botella"</formula1>
     </dataValidation>
   </dataValidations>
-  <pageMargins bottom="1" footer="0.5" header="0.5" left="0.75" right="0.75" top="1"/>
-  <pageSetup fitToHeight="0" fitToWidth="1" orientation="landscape"/>
+  <pageMargins left="0.59" right="0.59" top="0.59" bottom="0.59" header="0.3" footer="0.3"/>
+  <pageSetup orientation="landscape" paperSize="9" fitToHeight="0" fitToWidth="1"/>
+  <headerFooter>
+    <oddHeader/>
+    <oddFooter>&amp;C&amp;8 AI Chef Pro · aichef.pro · Página &amp;P de &amp;N</oddFooter>
+    <evenHeader/>
+    <evenFooter/>
+    <firstHeader/>
+    <firstFooter/>
+  </headerFooter>
 </worksheet>
 </file>
</xml_diff>